<commit_message>
& - 25929 от 27.01.2026 https://2eurostore.ru/
</commit_message>
<xml_diff>
--- a/Collections/EURO/Austria/#EURO#Austria#Commemorative#[2005-present]#UNC.xlsx
+++ b/Collections/EURO/Austria/#EURO#Austria#Commemorative#[2005-present]#UNC.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lord_Alexator\Documents\CoinCollection\Collections\EURO\Austria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B0056F4-59D0-42EF-8D6B-5EC7B61B9E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE39009-5622-4E07-9AFA-9648A58D90F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,6 +32,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1324,7 +1327,7 @@
         <v>29</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F20" s="9">
         <v>2590000</v>

</xml_diff>